<commit_message>
docs: add product and sprint backlog documentation, environment rules, and project tracking spreadsheet
</commit_message>
<xml_diff>
--- a/docs/Backlog_Barberia_v1.xlsx
+++ b/docs/Backlog_Barberia_v1.xlsx
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Cada servicio tiene nombre, duración (minutos) y precio.
+          <t>El servicio expone nombre, duración (minutos) y precio a través de su relación con `Item_Catalogo` (ver `glosario_datos.md`, entidades ITEM_CATALOGO y SERVICIO) — estos campos NO viven directamente en la tabla de Servicio.
 El precio es único por servicio (no varía por barbero).
 No se puede eliminar un servicio que ya tiene turnos históricos asociados (se desactiva en su lugar).</t>
         </is>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Debe existir un servicio (con duración) antes de poder agendar un turno.</t>
+          <t>Debe existir un servicio (con duración) antes de poder agendar un turno. **Incluye crear el modelo `Item_Catalogo`** (ver glosario_datos.md): Servicio no tiene nombre/precio/duración propios, los expone a través de Item_Catalogo. Toda HU posterior que toque Servicio o Combo (HU-TUR-04, HU-SER-02, HU-SER-03) asume que esta estructura ya está bien implementada.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update de los archivos
</commit_message>
<xml_diff>
--- a/docs/Backlog_Barberia_v1.xlsx
+++ b/docs/Backlog_Barberia_v1.xlsx
@@ -697,7 +697,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="80" customHeight="1">
+    <row r="6" ht="152" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>HU-TUR-02</t>
@@ -731,9 +731,13 @@
       <c r="G6" s="6" t="inlineStr">
         <is>
           <t>La página pública muestra únicamente los horarios disponibles, ya bloqueados según turnos existentes.
+Un horario cuenta como "disponible" solo si tiene espacio suficiente para la duración completa del servicio/combo elegido, sin invadir el siguiente turno ya agendado (más un margen de 5 minutos entre turnos — ver constante `TURNO_BUFFER_MINUTOS` o equivalente). Este cálculo debe rehacerse cada vez que cambia el servicio elegido, ya que la misma grilla de horarios puede tener distinta disponibilidad según la duración de cada servicio.
+Al confirmar una reserva, el horario recién tomado deja de listarse como disponible inmediatamente (sin necesidad de recargar la página manualmente) para evitar que otro cliente lo vea libre.
 El cliente elige un servicio y ve la duración antes de confirmar.
 Si el cliente no tiene cuenta, se lo dirige al flujo de autoregistro (HU-CLI-01) antes de confirmar.
-Al confirmar, el turno queda visible en la agenda del staff en tiempo real.</t>
+Al confirmar, el cliente es redirigido a una pantalla de confirmación/inicio (no permanece en el formulario de reserva).
+Al confirmar, el turno queda visible en la agenda del staff en tiempo real.
+La hora que el cliente selecciona y confirma en el frontend es exactamente la misma hora que queda guardada en fecha_hora_inicio y la que ve el staff en el dashboard — sin corrimientos por zona horaria en ningún punto de la cadena (selección → envío al backend → guardado en base → lectura desde el backend → visualización en el dashboard).</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">

</xml_diff>